<commit_message>
Improve Office2MD RAG extraction and Excel tables
Preserve diagram connections and slide position metadata, detect merged and named Excel table headers, and publish reproducible conversion examples.
</commit_message>
<xml_diff>
--- a/docs/APIDocs/office2md/examples/excel-complex/input.xlsx
+++ b/docs/APIDocs/office2md/examples/excel-complex/input.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="190">
   <si>
     <t>文章と書式の変換テスト</t>
   </si>
@@ -607,6 +607,9 @@
     <t>GRP05  背景図形＋PNG：図形と画像を別々に出力</t>
   </si>
   <si>
+    <t>GRP06  保存IDなし：線端が境界に接触する横・斜めの接続を1枚に統合</t>
+  </si>
+  <si>
     <t>07  未対応要素と加工の通知</t>
   </si>
   <si>
@@ -658,7 +661,7 @@
     <numFmt numFmtId="168" formatCode="hh:mm"/>
     <numFmt numFmtId="169" formatCode="#,##0;(#,##0)"/>
   </numFmts>
-  <fonts count="44">
+  <fonts count="45">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -873,6 +876,12 @@
     </font>
     <font>
       <name val="Noto Sans CJK JP"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color rgb="FF00828C"/>
+    </font>
+    <font>
+      <name val="Noto Sans CJK JP"/>
       <sz val="22.0"/>
       <b val="true"/>
       <color rgb="FF142941"/>
@@ -1008,7 +1017,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="center" wrapText="true"/>
@@ -1395,6 +1404,7 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment vertical="center" wrapText="true"/>
     </xf>
@@ -3407,6 +3417,262 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Shape 1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="4000500" cy="1828800"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="E9F1FB"/>
+        </a:solidFill>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="00828C"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr anchor="t" rtlCol="false" lIns="127000" rIns="101600" tIns="127000" bIns="101600"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="true">
+              <a:solidFill>
+                <a:srgbClr val="142941"/>
+              </a:solidFill>
+              <a:latin typeface="Noto Sans CJK JP" charset="0" pitchFamily="0"/>
+              <a:ea typeface="Noto Sans CJK JP"/>
+            </a:rPr>
+            <a:t>申請</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Shape 1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="4000500" cy="1828800"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="E7F6F5"/>
+        </a:solidFill>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="00828C"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr anchor="t" rtlCol="false" lIns="127000" rIns="101600" tIns="127000" bIns="101600"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="true">
+              <a:solidFill>
+                <a:srgbClr val="142941"/>
+              </a:solidFill>
+              <a:latin typeface="Noto Sans CJK JP" charset="0" pitchFamily="0"/>
+              <a:ea typeface="Noto Sans CJK JP"/>
+            </a:rPr>
+            <a:t>確認</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Shape 1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="3200400" cy="1828800"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="E9F1FB"/>
+        </a:solidFill>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="00828C"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr anchor="t" rtlCol="false" lIns="127000" rIns="101600" tIns="127000" bIns="101600"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="true">
+              <a:solidFill>
+                <a:srgbClr val="142941"/>
+              </a:solidFill>
+              <a:latin typeface="Noto Sans CJK JP" charset="0" pitchFamily="0"/>
+              <a:ea typeface="Noto Sans CJK JP"/>
+            </a:rPr>
+            <a:t>保管</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="1" name="Shape 1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="25400">
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="1" name="Shape 1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="25400">
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -4060,7 +4326,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -4084,7 +4350,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -4098,18 +4364,18 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="153" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="153" t="s">
+      <c r="B1" s="154" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="154" t="s">
+      <c r="A2" s="155" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="155" t="s">
+      <c r="B2" s="156" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5015,7 +5281,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A78"/>
   <sheetFormatPr defaultRowHeight="24.0" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="12.0" customWidth="true"/>
@@ -5068,6 +5334,11 @@
     <row r="62">
       <c r="A62" t="s" s="144">
         <v>175</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="145">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -5104,18 +5375,18 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="true">
-      <c r="A1" t="s" s="145">
-        <v>176</v>
+      <c r="A1" t="s" s="146">
+        <v>177</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="146">
-        <v>177</v>
+      <c r="A3" t="s" s="147">
+        <v>178</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B5" t="n" s="0">
         <v>12.0</v>
@@ -5123,7 +5394,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B6" t="n" s="0">
         <v>18.0</v>
@@ -5131,29 +5402,29 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B7" t="n" s="0">
         <v>25.0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="s" s="147">
-        <v>181</v>
-      </c>
-      <c r="G19" t="s" s="148">
+      <c r="A19" t="s" s="148">
         <v>182</v>
       </c>
-      <c r="N19" t="s" s="149">
+      <c r="G19" t="s" s="149">
         <v>183</v>
       </c>
+      <c r="N19" t="s" s="150">
+        <v>184</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" t="s" s="150">
-        <v>184</v>
-      </c>
-      <c r="J33" t="s" s="151">
+      <c r="A33" t="s" s="151">
         <v>185</v>
+      </c>
+      <c r="J33" t="s" s="152">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -5193,7 +5464,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish API docs and expand Office2MD examples
</commit_message>
<xml_diff>
--- a/docs/APIDocs/office2md/examples/excel-complex/input.xlsx
+++ b/docs/APIDocs/office2md/examples/excel-complex/input.xlsx
@@ -20,6 +20,10 @@
     <sheet name="取消線のみ" r:id="rId15" sheetId="12"/>
     <sheet name="罫線のみ" r:id="rId16" sheetId="13"/>
   </sheets>
+  <definedNames>
+    <definedName name="InventoryGrid">'02_罫線の表'!$A$4:$D$9</definedName>
+    <definedName name="CachedResultCells">'03_表示値と数式'!$A$17:$C$18</definedName>
+  </definedNames>
 </workbook>
 </file>
 

</xml_diff>